<commit_message>
Add alumni who are professors at Korean universities to the map
Requested after the 정규열 (POSTECH) alumni page: 임성인 (Pukyong),
황현규 (Jeonbuk), 우성화 (KENTECH) and 예대열 (Gachon) go in the master
sheet's 교수추가 tab now. From here on the alumni collection does this
itself: an alumnus whose stated position is professor at a Korean
university and who is not in the map yet becomes a new professor row
(identity_status alumni_page; the OpenAlex profile is matched on the
next resolve). Professors abroad stay in the alumni statistics only.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -578,6 +578,94 @@
       <c r="H1" s="3" t="inlineStr">
         <is>
           <t>메모</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>임성인</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Pukyong National University</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Associate Professor · 사용자 요청 10/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>황현규</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Jeonbuk National University</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Professor · 사용자 요청 10/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>우성화</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>KENTECH</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Professor (한국에너지공과대학교) · 사용자 요청 10/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>예대열</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gachon University</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Professor · 사용자 요청 10/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alumni cards: 'Name / E-mail / Career' under degree headings; 김준원 lab homepage; add 전누리
- 한지숙 lab alumni page uses labelled cards grouped by Ph.D. / M.S.
- 한국화학연구원 and other national institutes count as institute, not industry
- 전누리 (SNU Bioengineering) added to the master sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -587,16 +587,11 @@
           <t>임성인</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Pukyong National University</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Associate Professor · 사용자 요청 10/13</t>
@@ -609,16 +604,11 @@
           <t>황현규</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Jeonbuk National University</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Professor · 사용자 요청 10/13</t>
@@ -631,16 +621,11 @@
           <t>우성화</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>KENTECH</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Professor (한국에너지공과대학교) · 사용자 요청 10/13</t>
@@ -653,19 +638,41 @@
           <t>예대열</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Gachon University</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>정규열 교수 연구실(POSTECH) 졸업생 페이지: Professor · 사용자 요청 10/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>전누리</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Noo Li Jeon</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정 (기계공학부)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alumni: stated degree time ('석사 2년'), foreign names in Hangul, 'Our team' pages; add 안지완
- 송준명 lab lists the time per graduate; it is used as an exact duration
- probe: no positions printed; 'Name (Romanised)' and short Hangul lines masked
- 안지완 (SNU School of Dentistry) added to the master sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -671,6 +671,28 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>안지완</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>치의학대학원</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>사용자 요청 10/15</t>
         </is>

</xml_diff>

<commit_message>
Add 이연 and 이남기 (SNU Chemistry); probe the SNU Chemistry site for its faculty page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -693,6 +693,60 @@
         </is>
       </c>
       <c r="H7" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>이연</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Yan Lee</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>화학부</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>이남기</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Nam Ki Lee</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>화학부</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>사용자 요청 10/15</t>
         </is>

</xml_diff>

<commit_message>
Add 김교범 (Dongguk University) with lab homepage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -747,6 +747,33 @@
         </is>
       </c>
       <c r="H9" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>김교범</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kyobum Kim</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://kkim2014.wixsite.com/tissueeng</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>사용자 요청 10/15</t>
         </is>

</xml_diff>

<commit_message>
Add 박천권 (Sungkyunkwan University) with lab homepage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -774,6 +774,38 @@
         </is>
       </c>
       <c r="H10" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>박천권</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Chun Gwon Park</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/skkucbrl/</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>사용자 요청 10/15</t>
         </is>

</xml_diff>

<commit_message>
Add 임용택 (Sungkyunkwan University) with lab homepage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -806,6 +806,38 @@
         </is>
       </c>
       <c r="H11" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>임용택</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Yong Taik Lim</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>나노공학과</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/laboflim/home</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>사용자 요청 10/15</t>
         </is>

</xml_diff>

<commit_message>
Add 42 SNU Bioengineering faculty missing from the map
The department page links 56 professor profiles; the crawl had read 3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -840,6 +840,930 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>강승균</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>강준호</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>강홍기</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>고승환</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>권성훈</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>김경수</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>김도년</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>김영수</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>김성완</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>김영은</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>남기태</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>문민환</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>박종민</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>박주혁</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>박지웅</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>박창민</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>백남종</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>서종모</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>신상도</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>신용대</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>안철희</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>오세일</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>윤형진</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>이경호</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>이규언</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>이동헌</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>이상훈</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>이시욱</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>최진욱</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>이재성</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>이정렬</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>이정찬</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>이창한</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>이태우</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>임재영</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>정기영</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>정현훈</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>조규진</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>최승홍</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>최영빈</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>한경원</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>허찬영</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>바이오엔지니어링 협동과정</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Alumni links: Korean university names in positions; add 류주희 (KIST)
강미경 (Korea Univ.) and 홍지혜 (Dankook Univ.), 김병수 lab alumni added yesterday, appear
with today's publish and link to their advisor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1764,6 +1764,28 @@
       <c r="H54" t="inlineStr">
         <is>
           <t>서울대 바이오엔지니어링 교수진 목록 (https://bioeng.snu.ac.kr/교수진-목록/) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>류주희</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Ju Hee Ryu</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Korea Institute of Science and Technology</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15 (KIST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 정석 (Korea Univ.) and 방석영 (Dongguk); probe Dongguk sites for the biomedical engineering faculty page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H55"/>
+  <dimension ref="A1:H57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1786,6 +1786,55 @@
       <c r="H55" t="inlineStr">
         <is>
           <t>사용자 요청 10/15 (KIST)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>정석</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Seok Chung</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>기계공학부</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>방석영</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Dongguk Biomedical Engineering faculty (9 + 방석영) and the department list as a source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1835,6 +1835,204 @@
       <c r="H57" t="inlineStr">
         <is>
           <t>사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>김성민</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>권영은</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>정종섭</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>이수홍</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>서영권</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>김진식</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>양승훈</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>이승훈</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>홍영택</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>의생명공학과</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Dongguk Food Biotechnology faculty and the department list as a source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2033,6 +2033,204 @@
       <c r="H66" t="inlineStr">
         <is>
           <t>동국대 의생명공학과 교수진 목록 (life.dongguk.edu, PROFH_033) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>유병승</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>이광근</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>신한승</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>강석성</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>금나나</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>강준원</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>박유헌</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>이석희</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>김도영</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Dongguk University</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>식품생명공학과</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Korea University Biomedical Engineering faculty and the department list as a source
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2231,6 +2231,358 @@
       <c r="H75" t="inlineStr">
         <is>
           <t>동국대 식품생명공학과 교수진 목록 (life.dongguk.edu, PROFH_032) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>고영학</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>구자현</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>김법민</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>성준경</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>염정열</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>유용상</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>윤대성</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>윤명근</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>이규백</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>이기성</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>정아람</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>정하욱</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>정호상</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>천홍구</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>최연호</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>최영운</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Korea University</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>바이오의공학부</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
임용택 (SKKU) alumni page; add 김용호 (SKKU Nano Engineering) to the master sheet; probe masks bracketed romanised names; probe 김용호's lab site and OpenAlex profile
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2583,6 +2583,38 @@
       <c r="H91" t="inlineStr">
         <is>
           <t>고려대 바이오의공학부 교수진 (bmeng.korea.ac.kr) · 사용자 요청 10/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>김용호</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Yong Ho Kim</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>나노공학과</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://www.yhproteinlab.com/</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add SKKU Integrative Biotechnology (13) and Global Biomedical Engineering (19) faculty, and both department pages as sources; reset probe defaults
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H92"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2615,6 +2615,725 @@
       <c r="H92" t="inlineStr">
         <is>
           <t>사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>이석찬</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>권대혁</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>윤기정</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>조재열</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>오정수</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>정우재</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>이종성</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>송민경</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>전영준</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>김희권</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>발라찬드란마나발란</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Balachandran Manavalan</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>백가현</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>양유수</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>융합생명공학과</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>성균관대 융합생명공학과 교수진 (skb.skku.edu/gene) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>김병철</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>김재현</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>김태형</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>김형구</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>박장연</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>박재석</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>박진형</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>박한규</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>서민아</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>손한샘</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>신미경</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>심원목</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>아우렐리오코르테제</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Aurelio Cortese</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>우충완</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>유승범</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>이정승</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>이준열</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>학완라우</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Hakwan Lau</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>홍석준</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>글로벌바이오메디컬공학과</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 김근형 (SKKU) to the master sheet with his lab homepage
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H124"/>
+  <dimension ref="A1:H125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3334,6 +3334,33 @@
       <c r="H124" t="inlineStr">
         <is>
           <t>성균관대 글로벌바이오메디컬공학과 교수진 (skb.skku.edu/gbme) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>김근형</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Geun Hyung Kim</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>https://partsweb.skku.edu/~gkimbme/</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>사용자 요청 10/16 (3D 바이오프린팅·조직공학)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Master sheet: lineage lines 정규열→양진아 (PhD), 서상우→양진아 (postdoc), 서상우→한용희 (PhD); SKKU School of Medicine basic-science faculty (active, Suwon 의학관)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SSf7Q41rU8hNPx2LWVoT6C
</commit_message>
<xml_diff>
--- a/0. korea bio map/data/about_bio_master.xlsx
+++ b/0. korea bio map/data/about_bio_master.xlsx
@@ -526,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H125"/>
+  <dimension ref="A1:H170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3364,6 +3364,1076 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>강동묵</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>강종순</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>http://biomed.skku.edu/stemcell</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>고관수</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>http://biomed.skku.edu/medbact</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>권일민</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>김경규</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>김균환</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>김기주</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>https://biomedical.skku.edu/</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>김문영</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>김성태</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>김재준</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>김태진</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>김현진</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>남주현</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>류희주</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>문성지</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>밀롯미르디타</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Milot Mirdita</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>https://mirdita.org</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>박명규</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>박성진</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>박재현</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>배창대</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>백관혁</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>https://khbaek9.wixsite.com/biolab</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>신동우</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>http://biomed.skku.edu/molbact</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>신명희</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>신주호</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>https://biomed.skku.edu/jhshin</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>안지인</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>http://biomed.skku.edu/jeeahn</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>안진현</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>http://biomed.skku.edu/virology</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>엄성희</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>http://biomed.skku.edu/shum</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>오창석</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>원태형</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>이경훈</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>이성균</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>이승원</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/view/mbd-lab/</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>이연종</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>이윤송</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>이주상</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>https://leejoosang.wixsite.com/ngml</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>이창우</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>http://biomed.skku.edu/cwlee</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>임세진</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>전용현</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>정지욱</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>정지헌</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>https://jeeheon9.wixsite.com/jeong</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>정호창</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>조영석</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>조하나</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>주경민</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>https://sites.google.com/g.skku.edu/jool</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>최정윤</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Sungkyunkwan University</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>의과대학 (기초의학)</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>성균관대 의대 기초의학 현직 (professor.skku.edu, 수원 의학관) · 사용자 요청 10/16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3375,7 +4445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3421,6 +4491,102 @@
       <c r="G1" s="3" t="inlineStr">
         <is>
           <t>메모</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>정규열</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>POSTECH</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>양진아</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Jeju National University</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>지도교수-제자</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>사용자 제보 (10/16): 양진아 = 정규열 교수 박사</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>서상우</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>양진아</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Jeju National University</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>포닥멘토-포닥</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>사용자 제보 (10/16): 양진아 = 서상우 교수 포닥</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>서상우</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Seoul National University</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>한용희</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Chonnam National University</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>지도교수-제자</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>사용자 제보 (10/16): 한용희 = 서상우 교수 박사, 교수 배출</t>
         </is>
       </c>
     </row>

</xml_diff>